<commit_message>
files are placed in Scenario Selection Module
</commit_message>
<xml_diff>
--- a/SSTSS_GenSim_Modules/Scenario_Selection_Module/user_selected_scenarios_from_catalog.xlsx
+++ b/SSTSS_GenSim_Modules/Scenario_Selection_Module/user_selected_scenarios_from_catalog.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -59,13 +59,6 @@
       <name val="Calibri"/>
       <charset val="1"/>
       <family val="2"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Cambria"/>
-      <charset val="1"/>
-      <family val="0"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
@@ -134,13 +127,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -167,9 +160,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -198,10 +188,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -576,279 +563,279 @@
   <dimension ref="A1:AK69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.171875" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="8.529999999999999" customWidth="1" style="10" min="1" max="1"/>
-    <col width="37.73" customWidth="1" style="10" min="3" max="3"/>
-    <col width="30.53" customWidth="1" style="10" min="4" max="4"/>
-    <col width="8.529999999999999" customWidth="1" style="10" min="5" max="5"/>
-    <col width="15.54" customWidth="1" style="10" min="6" max="7"/>
-    <col width="15.17" customWidth="1" style="10" min="8" max="8"/>
-    <col width="8.529999999999999" customWidth="1" style="10" min="9" max="17"/>
-    <col width="21.28" customWidth="1" style="10" min="18" max="18"/>
-    <col width="19.55" customWidth="1" style="10" min="19" max="19"/>
-    <col width="18.55" customWidth="1" style="10" min="20" max="20"/>
-    <col width="30.18" customWidth="1" style="10" min="21" max="21"/>
-    <col width="6.27" customWidth="1" style="10" min="22" max="22"/>
-    <col width="21" customWidth="1" style="10" min="23" max="23"/>
-    <col width="19.55" customWidth="1" style="10" min="24" max="24"/>
-    <col width="13.17" customWidth="1" style="10" min="25" max="25"/>
-    <col width="17.72" customWidth="1" style="10" min="26" max="26"/>
-    <col width="15" customWidth="1" style="10" min="27" max="27"/>
-    <col width="13.45" customWidth="1" style="10" min="28" max="28"/>
-    <col width="15.72" customWidth="1" style="10" min="29" max="30"/>
-    <col width="11.45" customWidth="1" style="10" min="31" max="31"/>
-    <col width="10" customWidth="1" style="10" min="32" max="32"/>
-    <col width="23.18" customWidth="1" style="10" min="33" max="33"/>
-    <col width="22.45" customWidth="1" style="10" min="34" max="34"/>
-    <col width="16.45" customWidth="1" style="10" min="35" max="35"/>
-    <col width="59.42" customWidth="1" style="10" min="36" max="36"/>
-    <col width="8.529999999999999" customWidth="1" style="10" min="37" max="64"/>
+    <col width="8.529999999999999" customWidth="1" style="9" min="1" max="1"/>
+    <col width="37.73" customWidth="1" style="9" min="3" max="3"/>
+    <col width="30.53" customWidth="1" style="9" min="4" max="4"/>
+    <col width="8.529999999999999" customWidth="1" style="9" min="5" max="5"/>
+    <col width="15.54" customWidth="1" style="9" min="6" max="7"/>
+    <col width="15.17" customWidth="1" style="9" min="8" max="8"/>
+    <col width="8.529999999999999" customWidth="1" style="9" min="9" max="17"/>
+    <col width="21.28" customWidth="1" style="9" min="18" max="18"/>
+    <col width="19.55" customWidth="1" style="9" min="19" max="19"/>
+    <col width="18.55" customWidth="1" style="9" min="20" max="20"/>
+    <col width="30.18" customWidth="1" style="9" min="21" max="21"/>
+    <col width="6.27" customWidth="1" style="9" min="22" max="22"/>
+    <col width="21" customWidth="1" style="9" min="23" max="23"/>
+    <col width="19.55" customWidth="1" style="9" min="24" max="24"/>
+    <col width="13.17" customWidth="1" style="9" min="25" max="25"/>
+    <col width="17.72" customWidth="1" style="9" min="26" max="26"/>
+    <col width="15" customWidth="1" style="9" min="27" max="27"/>
+    <col width="13.45" customWidth="1" style="9" min="28" max="28"/>
+    <col width="15.72" customWidth="1" style="9" min="29" max="30"/>
+    <col width="11.45" customWidth="1" style="9" min="31" max="31"/>
+    <col width="10" customWidth="1" style="9" min="32" max="32"/>
+    <col width="23.18" customWidth="1" style="9" min="33" max="33"/>
+    <col width="22.45" customWidth="1" style="9" min="34" max="34"/>
+    <col width="16.45" customWidth="1" style="9" min="35" max="35"/>
+    <col width="59.42" customWidth="1" style="9" min="36" max="36"/>
+    <col width="8.529999999999999" customWidth="1" style="9" min="37" max="64"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" s="11">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="14.25" customHeight="1" s="10">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Scenario ID</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Actors</t>
         </is>
       </c>
-      <c r="F1" s="13" t="n"/>
-      <c r="G1" s="13" t="n"/>
-      <c r="H1" s="13" t="n"/>
-      <c r="I1" s="13" t="n"/>
-      <c r="J1" s="14" t="n"/>
-      <c r="K1" s="12" t="inlineStr">
+      <c r="F1" s="12" t="n"/>
+      <c r="G1" s="12" t="n"/>
+      <c r="H1" s="12" t="n"/>
+      <c r="I1" s="12" t="n"/>
+      <c r="J1" s="13" t="n"/>
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Weather</t>
         </is>
       </c>
-      <c r="L1" s="13" t="n"/>
-      <c r="M1" s="13" t="n"/>
-      <c r="N1" s="14" t="n"/>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="L1" s="12" t="n"/>
+      <c r="M1" s="12" t="n"/>
+      <c r="N1" s="13" t="n"/>
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="P1" s="13" t="n"/>
-      <c r="Q1" s="14" t="n"/>
-      <c r="R1" s="12" t="inlineStr">
+      <c r="P1" s="12" t="n"/>
+      <c r="Q1" s="13" t="n"/>
+      <c r="R1" s="11" t="inlineStr">
         <is>
           <t>Driving Maneuver</t>
         </is>
       </c>
-      <c r="S1" s="13" t="n"/>
-      <c r="T1" s="13" t="n"/>
-      <c r="U1" s="13" t="n"/>
-      <c r="V1" s="13" t="n"/>
-      <c r="W1" s="13" t="n"/>
-      <c r="X1" s="13" t="n"/>
-      <c r="Y1" s="13" t="n"/>
-      <c r="Z1" s="13" t="n"/>
-      <c r="AA1" s="13" t="n"/>
-      <c r="AB1" s="13" t="n"/>
-      <c r="AC1" s="13" t="n"/>
-      <c r="AD1" s="13" t="n"/>
-      <c r="AE1" s="13" t="n"/>
-      <c r="AF1" s="14" t="n"/>
-      <c r="AG1" s="12" t="inlineStr">
+      <c r="S1" s="12" t="n"/>
+      <c r="T1" s="12" t="n"/>
+      <c r="U1" s="12" t="n"/>
+      <c r="V1" s="12" t="n"/>
+      <c r="W1" s="12" t="n"/>
+      <c r="X1" s="12" t="n"/>
+      <c r="Y1" s="12" t="n"/>
+      <c r="Z1" s="12" t="n"/>
+      <c r="AA1" s="12" t="n"/>
+      <c r="AB1" s="12" t="n"/>
+      <c r="AC1" s="12" t="n"/>
+      <c r="AD1" s="12" t="n"/>
+      <c r="AE1" s="12" t="n"/>
+      <c r="AF1" s="13" t="n"/>
+      <c r="AG1" s="11" t="inlineStr">
         <is>
           <t>Road Topology</t>
         </is>
       </c>
-      <c r="AH1" s="13" t="n"/>
-      <c r="AI1" s="14" t="n"/>
-      <c r="AJ1" s="15" t="n"/>
-      <c r="AK1" s="15" t="inlineStr">
+      <c r="AH1" s="12" t="n"/>
+      <c r="AI1" s="13" t="n"/>
+      <c r="AJ1" s="14" t="n"/>
+      <c r="AK1" s="14" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1" s="11">
-      <c r="A2" s="12" t="inlineStr">
+    <row r="2" ht="14.25" customHeight="1" s="10">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n"/>
-      <c r="C2" s="12" t="n"/>
-      <c r="D2" s="12" t="n"/>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="B2" s="11" t="n"/>
+      <c r="C2" s="11" t="n"/>
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Vehicle</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Pedestrian</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>Motorcyclist</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>Pedal cyclist</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>Animal</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>Dry</t>
         </is>
       </c>
-      <c r="L2" s="12" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>Rain</t>
         </is>
       </c>
-      <c r="M2" s="12" t="inlineStr">
+      <c r="M2" s="11" t="inlineStr">
         <is>
           <t>Snow</t>
         </is>
       </c>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="N2" s="11" t="inlineStr">
         <is>
           <t>Fog</t>
         </is>
       </c>
-      <c r="O2" s="12" t="inlineStr">
+      <c r="O2" s="11" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="P2" s="12" t="inlineStr">
+      <c r="P2" s="11" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="Q2" s="12" t="inlineStr">
+      <c r="Q2" s="11" t="inlineStr">
         <is>
           <t>Twilight</t>
         </is>
       </c>
-      <c r="R2" s="12" t="inlineStr">
+      <c r="R2" s="11" t="inlineStr">
         <is>
           <t>Driving Straight</t>
         </is>
       </c>
-      <c r="S2" s="12" t="inlineStr">
+      <c r="S2" s="11" t="inlineStr">
         <is>
           <t>Negotiating a Curve</t>
         </is>
       </c>
-      <c r="T2" s="12" t="inlineStr">
+      <c r="T2" s="11" t="inlineStr">
         <is>
           <t>Turning Left</t>
         </is>
       </c>
-      <c r="U2" s="12" t="inlineStr">
+      <c r="U2" s="11" t="inlineStr">
         <is>
           <t>Passing or Overtaking Another Vehicle</t>
         </is>
       </c>
-      <c r="V2" s="12" t="inlineStr">
+      <c r="V2" s="11" t="inlineStr">
         <is>
           <t>Merging/Changing Lanes</t>
         </is>
       </c>
-      <c r="W2" s="12" t="inlineStr">
+      <c r="W2" s="11" t="inlineStr">
         <is>
           <t>Stopped in Roadway</t>
         </is>
       </c>
-      <c r="X2" s="12" t="inlineStr">
+      <c r="X2" s="11" t="inlineStr">
         <is>
           <t>Other Maneuver</t>
         </is>
       </c>
-      <c r="Y2" s="12" t="inlineStr">
+      <c r="Y2" s="11" t="inlineStr">
         <is>
           <t>Turning Right</t>
         </is>
       </c>
-      <c r="Z2" s="12" t="inlineStr">
+      <c r="Z2" s="11" t="inlineStr">
         <is>
           <t>Decelerating in Road</t>
         </is>
       </c>
-      <c r="AA2" s="12" t="inlineStr">
+      <c r="AA2" s="11" t="inlineStr">
         <is>
           <t>Starting in Road</t>
         </is>
       </c>
-      <c r="AB2" s="12" t="inlineStr">
+      <c r="AB2" s="11" t="inlineStr">
         <is>
           <t>Making a U-turn</t>
         </is>
       </c>
-      <c r="AC2" s="12" t="inlineStr">
+      <c r="AC2" s="11" t="inlineStr">
         <is>
           <t>Backing Up</t>
         </is>
       </c>
-      <c r="AD2" s="12" t="inlineStr">
+      <c r="AD2" s="11" t="inlineStr">
         <is>
           <t>Parked in Travel Lane</t>
         </is>
       </c>
-      <c r="AE2" s="12" t="inlineStr">
+      <c r="AE2" s="11" t="inlineStr">
         <is>
           <t>Leaving a Parking Position</t>
         </is>
       </c>
-      <c r="AF2" s="12" t="inlineStr">
+      <c r="AF2" s="11" t="inlineStr">
         <is>
           <t>Entering a Parking Position</t>
         </is>
       </c>
-      <c r="AG2" s="12" t="inlineStr">
+      <c r="AG2" s="11" t="inlineStr">
         <is>
           <t>With Signalized Junction</t>
         </is>
       </c>
-      <c r="AH2" s="12" t="inlineStr">
+      <c r="AH2" s="11" t="inlineStr">
         <is>
           <t>Non-Signalized Junction</t>
         </is>
       </c>
-      <c r="AI2" s="12" t="inlineStr">
+      <c r="AI2" s="11" t="inlineStr">
         <is>
           <t>Non-Junction</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1" s="11">
+    <row r="3" ht="14.25" customHeight="1" s="10">
       <c r="A3" t="n">
         <v>1</v>
       </c>
@@ -972,7 +959,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1" s="11">
+    <row r="4" ht="14.25" customHeight="1" s="10">
       <c r="A4" t="n">
         <v>1</v>
       </c>
@@ -1095,7 +1082,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="14.25" customHeight="1" s="11">
+    <row r="5" ht="14.25" customHeight="1" s="10">
       <c r="A5" t="n">
         <v>2</v>
       </c>
@@ -1218,7 +1205,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="14.25" customHeight="1" s="11">
+    <row r="6" ht="14.25" customHeight="1" s="10">
       <c r="A6" t="n">
         <v>3</v>
       </c>
@@ -1341,7 +1328,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="14.25" customHeight="1" s="11">
+    <row r="7" ht="14.25" customHeight="1" s="10">
       <c r="A7" t="n">
         <v>4</v>
       </c>
@@ -1464,7 +1451,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="14.25" customHeight="1" s="11">
+    <row r="8" ht="14.25" customHeight="1" s="10">
       <c r="A8" t="n">
         <v>5</v>
       </c>
@@ -1587,7 +1574,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="14.25" customHeight="1" s="11">
+    <row r="9" ht="14.25" customHeight="1" s="10">
       <c r="A9" t="n">
         <v>6</v>
       </c>
@@ -1710,7 +1697,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="14.25" customHeight="1" s="11">
+    <row r="10" ht="14.25" customHeight="1" s="10">
       <c r="A10" t="n">
         <v>7</v>
       </c>
@@ -1833,7 +1820,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="14.25" customHeight="1" s="11">
+    <row r="11" ht="14.25" customHeight="1" s="10">
       <c r="A11" t="n">
         <v>8</v>
       </c>
@@ -1956,7 +1943,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="14.25" customHeight="1" s="11">
+    <row r="12" ht="14.25" customHeight="1" s="10">
       <c r="A12" t="n">
         <v>9</v>
       </c>
@@ -2079,7 +2066,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="14.25" customHeight="1" s="11">
+    <row r="13" ht="14.25" customHeight="1" s="10">
       <c r="A13" t="n">
         <v>10</v>
       </c>
@@ -2202,7 +2189,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="14.25" customHeight="1" s="11">
+    <row r="14" ht="14.25" customHeight="1" s="10">
       <c r="A14" t="n">
         <v>11</v>
       </c>
@@ -2325,7 +2312,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="14.25" customHeight="1" s="11">
+    <row r="15" ht="14.25" customHeight="1" s="10">
       <c r="A15" t="n">
         <v>12</v>
       </c>
@@ -2448,7 +2435,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="14.25" customHeight="1" s="11">
+    <row r="16" ht="14.25" customHeight="1" s="10">
       <c r="A16" t="n">
         <v>13</v>
       </c>
@@ -2571,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1" s="11">
+    <row r="17" ht="14.25" customHeight="1" s="10">
       <c r="A17" t="n">
         <v>14</v>
       </c>
@@ -2694,7 +2681,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="14.25" customHeight="1" s="11">
+    <row r="18" ht="14.25" customHeight="1" s="10">
       <c r="A18" t="n">
         <v>15</v>
       </c>
@@ -2817,7 +2804,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="14.25" customHeight="1" s="11">
+    <row r="19" ht="14.25" customHeight="1" s="10">
       <c r="A19" t="n">
         <v>16</v>
       </c>
@@ -2940,7 +2927,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="14.25" customHeight="1" s="11">
+    <row r="20" ht="14.25" customHeight="1" s="10">
       <c r="A20" t="n">
         <v>17</v>
       </c>
@@ -3063,7 +3050,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="14.25" customHeight="1" s="11">
+    <row r="21" ht="14.25" customHeight="1" s="10">
       <c r="A21" t="n">
         <v>18</v>
       </c>
@@ -3186,7 +3173,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="14.25" customHeight="1" s="11">
+    <row r="22" ht="14.25" customHeight="1" s="10">
       <c r="A22" t="n">
         <v>19</v>
       </c>
@@ -3309,7 +3296,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="14.25" customHeight="1" s="11">
+    <row r="23" ht="14.25" customHeight="1" s="10">
       <c r="A23" t="n">
         <v>20</v>
       </c>
@@ -3432,7 +3419,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="14.25" customHeight="1" s="11">
+    <row r="24" ht="14.25" customHeight="1" s="10">
       <c r="A24" t="n">
         <v>21</v>
       </c>
@@ -3555,7 +3542,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="14.25" customHeight="1" s="11">
+    <row r="25" ht="14.25" customHeight="1" s="10">
       <c r="A25" t="n">
         <v>22</v>
       </c>
@@ -3678,7 +3665,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="14.25" customHeight="1" s="11">
+    <row r="26" ht="14.25" customHeight="1" s="10">
       <c r="A26" t="n">
         <v>23</v>
       </c>
@@ -3801,7 +3788,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="14.25" customHeight="1" s="11">
+    <row r="27" ht="14.25" customHeight="1" s="10">
       <c r="A27" t="n">
         <v>24</v>
       </c>
@@ -3924,7 +3911,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="14.25" customHeight="1" s="11">
+    <row r="28" ht="14.25" customHeight="1" s="10">
       <c r="A28" t="n">
         <v>25</v>
       </c>
@@ -4047,7 +4034,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="14.25" customHeight="1" s="11">
+    <row r="29" ht="14.25" customHeight="1" s="10">
       <c r="A29" t="n">
         <v>26</v>
       </c>
@@ -4170,7 +4157,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="14.25" customHeight="1" s="11">
+    <row r="30" ht="14.25" customHeight="1" s="10">
       <c r="A30" t="n">
         <v>27</v>
       </c>
@@ -4294,7 +4281,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="14.25" customHeight="1" s="11">
+    <row r="31" ht="14.25" customHeight="1" s="10">
       <c r="A31" t="n">
         <v>28</v>
       </c>
@@ -4417,7 +4404,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="14.25" customHeight="1" s="11">
+    <row r="32" ht="14.25" customHeight="1" s="10">
       <c r="A32" t="n">
         <v>29</v>
       </c>
@@ -4541,7 +4528,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="14.25" customHeight="1" s="11">
+    <row r="33" ht="14.25" customHeight="1" s="10">
       <c r="A33" t="n">
         <v>30</v>
       </c>
@@ -4665,7 +4652,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="14.25" customHeight="1" s="11">
+    <row r="34" ht="14.25" customHeight="1" s="10">
       <c r="A34" t="n">
         <v>31</v>
       </c>
@@ -4789,7 +4776,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="14.25" customHeight="1" s="11">
+    <row r="35" ht="14.25" customHeight="1" s="10">
       <c r="A35" t="n">
         <v>32</v>
       </c>
@@ -4913,7 +4900,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="14.25" customHeight="1" s="11">
+    <row r="36" ht="14.25" customHeight="1" s="10">
       <c r="A36" t="n">
         <v>33</v>
       </c>
@@ -5037,7 +5024,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="14.25" customHeight="1" s="11">
+    <row r="37" ht="14.25" customHeight="1" s="10">
       <c r="A37" t="n">
         <v>34</v>
       </c>
@@ -5161,7 +5148,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="14.25" customHeight="1" s="11">
+    <row r="38" ht="14.25" customHeight="1" s="10">
       <c r="A38" t="n">
         <v>35</v>
       </c>
@@ -5284,7 +5271,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="14.25" customHeight="1" s="11">
+    <row r="39" ht="14.25" customHeight="1" s="10">
       <c r="A39" t="n">
         <v>36</v>
       </c>
@@ -5407,7 +5394,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="14.25" customHeight="1" s="11">
+    <row r="40" ht="14.25" customHeight="1" s="10">
       <c r="A40" t="n">
         <v>37</v>
       </c>
@@ -5530,7 +5517,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="14.25" customHeight="1" s="11">
+    <row r="41" ht="14.25" customHeight="1" s="10">
       <c r="A41" t="n">
         <v>38</v>
       </c>
@@ -5653,7 +5640,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="14.25" customHeight="1" s="11">
+    <row r="42" ht="14.25" customHeight="1" s="10">
       <c r="A42" t="n">
         <v>39</v>
       </c>
@@ -5776,7 +5763,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="14.25" customHeight="1" s="11">
+    <row r="43" ht="14.25" customHeight="1" s="10">
       <c r="A43" t="n">
         <v>40</v>
       </c>
@@ -5900,7 +5887,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="14.25" customHeight="1" s="11">
+    <row r="44" ht="14.25" customHeight="1" s="10">
       <c r="A44" t="n">
         <v>41</v>
       </c>
@@ -6027,7 +6014,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="14.25" customHeight="1" s="11">
+    <row r="45" ht="14.25" customHeight="1" s="10">
       <c r="A45" t="n">
         <v>42</v>
       </c>
@@ -6152,7 +6139,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="14.25" customHeight="1" s="11">
+    <row r="46" ht="14.25" customHeight="1" s="10">
       <c r="A46" t="n">
         <v>43</v>
       </c>
@@ -6277,7 +6264,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="14.25" customHeight="1" s="11">
+    <row r="47" ht="14.25" customHeight="1" s="10">
       <c r="A47" t="n">
         <v>44</v>
       </c>
@@ -6401,7 +6388,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="14.25" customHeight="1" s="11">
+    <row r="48" ht="14.25" customHeight="1" s="10">
       <c r="A48" t="n">
         <v>45</v>
       </c>
@@ -6526,7 +6513,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="14.25" customHeight="1" s="11">
+    <row r="49" ht="14.25" customHeight="1" s="10">
       <c r="A49" t="n">
         <v>46</v>
       </c>
@@ -6654,7 +6641,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="14.25" customHeight="1" s="11">
+    <row r="50" ht="14.25" customHeight="1" s="10">
       <c r="A50" t="n">
         <v>47</v>
       </c>
@@ -6782,7 +6769,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="14.25" customHeight="1" s="11">
+    <row r="51" ht="14.25" customHeight="1" s="10">
       <c r="A51" t="n">
         <v>48</v>
       </c>
@@ -6911,7 +6898,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="14.25" customHeight="1" s="11">
+    <row r="52" ht="14.25" customHeight="1" s="10">
       <c r="A52" t="n">
         <v>49</v>
       </c>
@@ -7039,7 +7026,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="14.25" customHeight="1" s="11">
+    <row r="53" ht="14.25" customHeight="1" s="10">
       <c r="A53" t="n">
         <v>50</v>
       </c>
@@ -7164,7 +7151,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="14.25" customHeight="1" s="11">
+    <row r="54" ht="14.25" customHeight="1" s="10">
       <c r="A54" t="n">
         <v>51</v>
       </c>
@@ -7289,7 +7276,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="14.25" customHeight="1" s="11">
+    <row r="55" ht="14.25" customHeight="1" s="10">
       <c r="A55" t="n">
         <v>52</v>
       </c>
@@ -7414,7 +7401,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="14.25" customHeight="1" s="11">
+    <row r="56" ht="14.25" customHeight="1" s="10">
       <c r="A56" t="n">
         <v>53</v>
       </c>
@@ -7539,7 +7526,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="14.25" customHeight="1" s="11">
+    <row r="57" ht="14.25" customHeight="1" s="10">
       <c r="A57" t="n">
         <v>54</v>
       </c>
@@ -7665,7 +7652,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="14.25" customHeight="1" s="11">
+    <row r="58" ht="14.25" customHeight="1" s="10">
       <c r="A58" t="n">
         <v>55</v>
       </c>
@@ -7791,7 +7778,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="14.25" customHeight="1" s="11">
+    <row r="59" ht="14.25" customHeight="1" s="10">
       <c r="A59" t="n">
         <v>56</v>
       </c>
@@ -7916,7 +7903,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="14.25" customHeight="1" s="11">
+    <row r="60" ht="14.25" customHeight="1" s="10">
       <c r="A60" t="n">
         <v>57</v>
       </c>
@@ -8041,7 +8028,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="14.25" customHeight="1" s="11">
+    <row r="61" ht="14.25" customHeight="1" s="10">
       <c r="A61" t="n">
         <v>58</v>
       </c>
@@ -8169,7 +8156,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="14.25" customHeight="1" s="11">
+    <row r="62" ht="14.25" customHeight="1" s="10">
       <c r="A62" t="n">
         <v>59</v>
       </c>
@@ -8297,7 +8284,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="14.25" customHeight="1" s="11">
+    <row r="63" ht="14.25" customHeight="1" s="10">
       <c r="A63" t="n">
         <v>60</v>
       </c>
@@ -8425,7 +8412,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="14.25" customHeight="1" s="11">
+    <row r="64" ht="14.25" customHeight="1" s="10">
       <c r="A64" t="n">
         <v>61</v>
       </c>
@@ -8553,7 +8540,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="14.25" customHeight="1" s="11">
+    <row r="65" ht="14.25" customHeight="1" s="10">
       <c r="A65" t="n">
         <v>62</v>
       </c>
@@ -8678,7 +8665,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="14.25" customHeight="1" s="11">
+    <row r="66" ht="14.25" customHeight="1" s="10">
       <c r="A66" t="n">
         <v>63</v>
       </c>
@@ -8803,7 +8790,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="14.25" customHeight="1" s="11">
+    <row r="67" ht="14.25" customHeight="1" s="10">
       <c r="A67" t="n">
         <v>64</v>
       </c>
@@ -8926,7 +8913,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="14.25" customHeight="1" s="11">
+    <row r="68" ht="14.25" customHeight="1" s="10">
       <c r="A68" t="n">
         <v>65</v>
       </c>
@@ -9051,7 +9038,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="14.25" customHeight="1" s="11">
+    <row r="69" ht="14.25" customHeight="1" s="10">
       <c r="A69" t="n">
         <v>66</v>
       </c>
@@ -9176,23 +9163,25 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="14.25" customHeight="1" s="11"/>
-    <row r="71" ht="14.25" customHeight="1" s="11"/>
-    <row r="72" ht="14.25" customHeight="1" s="11"/>
-    <row r="1048563" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048564" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048565" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048566" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048567" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048568" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048569" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048570" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048571" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048572" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048573" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048574" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048575" ht="12.8" customHeight="1" s="11"/>
-    <row r="1048576" ht="12.8" customHeight="1" s="11"/>
+    <row r="1048558" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048559" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048560" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048561" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048562" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048563" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048564" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048565" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048566" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048567" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048568" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048569" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048570" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048571" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048572" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048573" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048574" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048575" ht="12.8" customHeight="1" s="10"/>
+    <row r="1048576" ht="12.8" customHeight="1" s="10"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="E1:J1"/>

</xml_diff>